<commit_message>
Update of read me and documentation to describe the catch dataset an update of the catch data up to 2024
</commit_message>
<xml_diff>
--- a/inputs/data/metadata_configuration_file.xlsx
+++ b/inputs/data/metadata_configuration_file.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-analysis\iotc-tcac-simulations\inputs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99E9B9A5-2AB0-403E-93EE-2883621A3EB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A2A89FB-3588-4CCA-BC2B-6AD80288866D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{285539CB-9A0C-4AA0-B324-24EFEBF5A269}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="64">
   <si>
     <t>Field name</t>
   </si>
@@ -87,18 +87,6 @@
     <t>YEAR</t>
   </si>
   <si>
-    <t>FLAG_CODE</t>
-  </si>
-  <si>
-    <t>FLEET_CODE</t>
-  </si>
-  <si>
-    <t>FISHERY_TYPE</t>
-  </si>
-  <si>
-    <t>FISHERY_CODE</t>
-  </si>
-  <si>
     <t>SCHOOL_TYPE_CODE</t>
   </si>
   <si>
@@ -114,42 +102,24 @@
     <t>Gregorian calendar year of the fishing activities</t>
   </si>
   <si>
-    <t>EUR.FRA</t>
-  </si>
-  <si>
     <t>Code List</t>
   </si>
   <si>
     <t>Classification to define the scale of the fishing operations, separating fisheries composed of vessels less than 24 m and operating exclusively in National Jurisdiction Areas (ART = Artisanal/coastal) and surface and longline fisheries that may operate on the High Seas (IND = Industrial)</t>
   </si>
   <si>
-    <t xml:space="preserve">Fishing gear used to catch the fish. GI = gillnets; HL = handlines; LL = longlines; OT = other gears; PL = pole-and-lines; PS = purse seines; TL = trolling lines </t>
-  </si>
-  <si>
     <t>IND</t>
   </si>
   <si>
     <t>PS</t>
   </si>
   <si>
-    <t>Behavioural or environmental context in which fishing activity occurs, particularly in purse seine and other surface fisheries. FS = free-swimming schools; LS = schools associated with drifting floating objects</t>
-  </si>
-  <si>
     <t>NJA_SYC</t>
   </si>
   <si>
     <t>YFT</t>
   </si>
   <si>
-    <t>Amount of fish caught and retained in live-weight equivalent (metric tonnes)</t>
-  </si>
-  <si>
-    <t>Area of origin of the catch, either the high seas (HIGH_SEAS) or the national jurisdiction areas identified with the ISO 3166 alpha-3 code of the country, except for the Chagos archipelago (CHAGOS) and France Overseas territory (FRAT)</t>
-  </si>
-  <si>
-    <t>ASFIS alpha-3 code of the fish species</t>
-  </si>
-  <si>
     <t>https://data.iotc.org/reference/latest/domain/legacy/#fisheryTypes</t>
   </si>
   <si>
@@ -159,21 +129,9 @@
     <t>FS</t>
   </si>
   <si>
-    <t>https://data.iotc.org/reference/latest/domain/legacy/#species</t>
-  </si>
-  <si>
-    <t>https://data.iotc.org/reference/latest/domain/legacy/#fleets</t>
-  </si>
-  <si>
     <t>EUR</t>
   </si>
   <si>
-    <t>Similar to flag code except in the case of European Union countries (EUR)</t>
-  </si>
-  <si>
-    <t>Flag state of the fishery vessels, combining the CPC in the case of European Union Member States and aggregating all non-CPCs as others (OTH) or not elsewhere included (NEI)</t>
-  </si>
-  <si>
     <t>ISO3_CODE</t>
   </si>
   <si>
@@ -211,6 +169,66 @@
   </si>
   <si>
     <t>Surface area (in square kilometres) of the NJA within the Indian Ocean</t>
+  </si>
+  <si>
+    <t>FISHERY_TYPE_CODE</t>
+  </si>
+  <si>
+    <t>GEAR_CODE</t>
+  </si>
+  <si>
+    <t>Fishing gear used to catch the fish</t>
+  </si>
+  <si>
+    <t>https://data.iotc.org/reference/latest/domain/legacy/#gears</t>
+  </si>
+  <si>
+    <t>ENTITY_CODE</t>
+  </si>
+  <si>
+    <t>https://data.iotc.org/reference/latest/domain/admin/#CPCs</t>
+  </si>
+  <si>
+    <t>https://data.iotc.org/reference/latest/domain/admin/#countries</t>
+  </si>
+  <si>
+    <t>Amount of fish caught and retained in live-weight equivalent, expressed in metric tonnes</t>
+  </si>
+  <si>
+    <t>ASFIS alpha-3 code identifying the species: ALB (albacore), BET (bigeye tuna), SKJ (skipjack tuna), SWO (swordfish), YFT (yellowfin tuna)</t>
+  </si>
+  <si>
+    <t>https://data.iotc.org/reference/latest/domain/biology/#IOTCspecies</t>
+  </si>
+  <si>
+    <t>Code identifying the type of tuna school association: LS = school associated with a drifting floating object, natural or artificial; FS = free-swimming school; UNCL = unclassified</t>
+  </si>
+  <si>
+    <t>Entity</t>
+  </si>
+  <si>
+    <t>Gear</t>
+  </si>
+  <si>
+    <t>Species</t>
+  </si>
+  <si>
+    <t>Type of fishery</t>
+  </si>
+  <si>
+    <t>Type of school</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Area where the catch is assigned. Values include Areas Beyond National Jurisdiction (HIGH_SEAS) and NJAs, where the last three characters correspond to the relevant country code, or the European Union (EUR) in the case of France. NJA_OTH represents all non-IOTC coastal States of the Indian Ocean</t>
+  </si>
+  <si>
+    <t>Code identifying the entity, i.e., CPC or the fishing fleet of Taiwan,China (TWN)</t>
+  </si>
+  <si>
+    <t>Code List Url</t>
   </si>
 </sst>
 </file>
@@ -251,7 +269,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -262,14 +280,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -626,10 +641,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>10</v>
@@ -640,7 +655,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>11</v>
@@ -651,7 +666,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
@@ -662,7 +677,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>12</v>
@@ -673,7 +688,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>13</v>
@@ -681,10 +696,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C7" s="2" t="b">
         <v>1</v>
@@ -692,10 +707,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="C8" s="2" t="b">
         <v>0</v>
@@ -706,7 +721,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="C9" s="2" t="b">
         <v>1</v>
@@ -717,7 +732,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="C10" s="2" t="b">
         <v>1</v>
@@ -728,9 +743,9 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
-      </c>
-      <c r="C11" s="6">
+        <v>43</v>
+      </c>
+      <c r="C11" s="4">
         <v>930250</v>
       </c>
     </row>
@@ -741,17 +756,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A5299DC-178B-4681-AD4A-DBFFBD3062EA}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.42578125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="82.42578125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="22.28515625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="66.42578125" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="31.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="105.140625" style="1" customWidth="1"/>
+    <col min="3" max="4" width="22.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="66.42578125" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>14</v>
       </c>
@@ -762,127 +777,141 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C2" s="3">
         <v>1995</v>
       </c>
-      <c r="D2" s="1"/>
-    </row>
-    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="D2" s="3"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="B6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D3" s="1"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="D7" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="B8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8" s="1"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="B9" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" s="3">
+        <v>51</v>
+      </c>
+      <c r="C9" s="5">
         <v>5200</v>
       </c>
-      <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C11" s="5"/>
+      <c r="D9" s="5"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>